<commit_message>
feat(projects): add IUS HydroGen micro-hydroelectric campus turbine project
</commit_message>
<xml_diff>
--- a/data/projects.xlsx
+++ b/data/projects.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ6"/>
+  <dimension ref="A1:AZ7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1906,6 +1906,244 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ius-hydro-plant</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="b">
+        <v>1</v>
+      </c>
+      <c r="D7" t="b">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Yenilenebilir Enerji &amp; Donanım İnovasyonu</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Renewable Energy &amp; Hardware Innovation</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Proje Fikri</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Project Idea</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Öneri</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Proposal</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>IUS HydroGen (Kampüs Mikro Hidroelektrik Santrali)</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>IUS HydroGen (Campus Micro-Hydroelectric Turbine)</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Kampüs arazisinden geçen nehirden su türbini ile temiz enerji üretimi ve otonom akıllı depolama hedefi.</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Generating clean campus energy and autonomous smart storage from the campus river via a micro water turbine.</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Bekir Enes Çokbekler (Sayman / Finans)</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Bekir Enes Çokbekler (Proje Lideri &amp; Finans)</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Bekir Enes Çokbekler (Project Lead &amp; Finance)</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>FENS Mühendislik Öğrencileri &amp; Araştırmacılar</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>FENS Engineering Students &amp; Researchers</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>./assets/hydro_plant_hero.webp</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>photorealistic concept render of a sleek university campus micro-hydroelectric water turbine installed in a gentle natural stream beside modern university buildings, cylindrical hydro turbine mechanism with dark graphite metal finish and subtle warm gold accent lighting, compact weatherproof battery storage enclosure on the stone riverbank, cinematic dusk lighting, modern campus architecture in background, shallow depth of field, 16:9, no text, no logos, no watermark, no identifiable faces</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>IUS Kampüsü Nehir Tipi Mikro Hidroelektrik Santrali Konsept Tasarımı</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>Concept render of IUS Campus Micro-Hydroelectric Power Turbine along the river</t>
+        </is>
+      </c>
+      <c r="AA7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>Kampüs içerisindeki öğrenci projeleri ve açık alan prototipleri için bağımsız, sürdürülebilir yeşil enerji kaynağı eksikliği ve nehir akış potansiyelinin değerlendirilememesi.</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>Lack of autonomous, off-grid sustainable energy sources for outdoor campus projects and student hardware prototypes, leaving the university's natural river flow unutilized.</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>Kampüs arazisinden geçen nehre yerleştirilecek yaklaşık 50 cm çapında ve 1 metre uzunluğunda mikro su değirmeni ve jeneratör mekanizması ile elektrik üretilmesi; akıllı konumlandırma yazılımı ve enerji depolama ünitesiyle kulüp projelerine ve çevre aydınlatmasına temiz güç sağlanması hedeflenmektedir.</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>Proposed deployment of a micro water turbine (~50cm diameter, 1m length) and generator along the campus river, equipped with dynamic flow-positioning firmware and battery storage to power student hardware and outdoor lighting.</t>
+        </is>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>IUS Rektörlüğü ve FENS Dekanlığı ile görüşülerek nehir kullanım izinlerinin alınması, su debi rejiminin ölçülmesi ve prototip şasi tasarımı için çalışma ekibinin kurulması planlanmaktadır.</t>
+        </is>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>Schedule preliminary briefing with IUS Rectorate and FENS Deanship for site permissions, conduct hydrologic flow measurements, and assemble the multidisciplinary student mechanical &amp; electrical team.</t>
+        </is>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>Türbin / Mekanik</t>
+        </is>
+      </c>
+      <c r="AI7" t="inlineStr">
+        <is>
+          <t>Turbine / Mechanics</t>
+        </is>
+      </c>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>50cm x 1m Silindirik Çark / Redüktör</t>
+        </is>
+      </c>
+      <c r="AK7" t="inlineStr">
+        <is>
+          <t>50cm x 1m Cylindrical Impeller / Gearbox</t>
+        </is>
+      </c>
+      <c r="AL7" t="inlineStr">
+        <is>
+          <t>Jeneratör &amp; Güç</t>
+        </is>
+      </c>
+      <c r="AM7" t="inlineStr">
+        <is>
+          <t>Generator &amp; Power</t>
+        </is>
+      </c>
+      <c r="AN7" t="inlineStr">
+        <is>
+          <t>AC/DC Alternatör &amp; MPPT Şarj Devresi</t>
+        </is>
+      </c>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>AC/DC Alternator &amp; MPPT Charge Controller</t>
+        </is>
+      </c>
+      <c r="AP7" t="inlineStr">
+        <is>
+          <t>Kontrol &amp; Yazılım</t>
+        </is>
+      </c>
+      <c r="AQ7" t="inlineStr">
+        <is>
+          <t>Control &amp; Software</t>
+        </is>
+      </c>
+      <c r="AR7" t="inlineStr">
+        <is>
+          <t>ESP32 / Otonom Akış Takip Yazılımı</t>
+        </is>
+      </c>
+      <c r="AS7" t="inlineStr">
+        <is>
+          <t>ESP32 / Autonomous Flow-Tracking Firmware</t>
+        </is>
+      </c>
+      <c r="AT7" t="inlineStr">
+        <is>
+          <t>Enerji Depolama</t>
+        </is>
+      </c>
+      <c r="AU7" t="inlineStr">
+        <is>
+          <t>Energy Storage</t>
+        </is>
+      </c>
+      <c r="AV7" t="inlineStr">
+        <is>
+          <t>LiFePO4 Batarya Paketi / BMS</t>
+        </is>
+      </c>
+      <c r="AW7" t="inlineStr">
+        <is>
+          <t>LiFePO4 Battery Bank / BMS Protection</t>
+        </is>
+      </c>
+      <c r="AX7" t="inlineStr"/>
+      <c r="AY7" t="inlineStr">
+        <is>
+          <t>urban-loft</t>
+        </is>
+      </c>
+      <c r="AZ7" t="inlineStr">
+        <is>
+          <t>./assets/hydro_plant_hero.webp</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>